<commit_message>
Deploy schematics files from 10991598b93f573c0fee88c6be0f004f2e3a8ddb
</commit_message>
<xml_diff>
--- a/web/schematics/BoM/Generic/m5-pantilt-bom.xlsx
+++ b/web/schematics/BoM/Generic/m5-pantilt-bom.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="164">
   <si>
     <t>Row</t>
   </si>
@@ -146,6 +146,15 @@
     <t>5</t>
   </si>
   <si>
+    <t>mountinghole_M2_M3</t>
+  </si>
+  <si>
+    <t>Hole1 Hole2 Hole3 Hole4</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
     <t>Generic connector, single row, 01x02, script generated (kicad-library-utils/schlib/autogen/connector/)</t>
   </si>
   <si>
@@ -167,7 +176,7 @@
     <t>C20079</t>
   </si>
   <si>
-    <t>6</t>
+    <t>7</t>
   </si>
   <si>
     <t>J5</t>
@@ -182,7 +191,7 @@
     <t>C2319</t>
   </si>
   <si>
-    <t>7</t>
+    <t>8</t>
   </si>
   <si>
     <t>Generic connector, single row, 01x03, script generated (kicad-library-utils/schlib/autogen/connector/)</t>
@@ -197,7 +206,7 @@
     <t>JST_EH_B3B-EH-A_1x03_P2.50mm_Vertical</t>
   </si>
   <si>
-    <t>8</t>
+    <t>9</t>
   </si>
   <si>
     <t>Generic connector, single row, 01x04, script generated (kicad-library-utils/schlib/autogen/connector/)</t>
@@ -215,7 +224,7 @@
     <t>https://www.sengoku.co.jp/mod/sgk_cart/detail.php?code=EEHD-55FC</t>
   </si>
   <si>
-    <t>9</t>
+    <t>10</t>
   </si>
   <si>
     <t>Generic connector, double row, 02x15, odd/even pin numbering scheme (row 1 odd numbers, row 2 even numbers), script generated (kicad-library-utils/schlib/autogen/connector/)</t>
@@ -233,7 +242,7 @@
     <t>https://www.switch-science.com/catalog/3654/</t>
   </si>
   <si>
-    <t>10</t>
+    <t>11</t>
   </si>
   <si>
     <t>J2</t>
@@ -242,7 +251,7 @@
     <t>PinSocket_2x15_P2.54mm_Vertical_SMD</t>
   </si>
   <si>
-    <t>11</t>
+    <t>12</t>
   </si>
   <si>
     <t>0.1A Ic, 45V Vce, PNP Transistor, SOT-23</t>
@@ -263,7 +272,7 @@
     <t>C2139</t>
   </si>
   <si>
-    <t>12</t>
+    <t>13</t>
   </si>
   <si>
     <t>-3.7A Id, -20V Vds, 65mOhm Rds, P-Channel HEXFET Power MOSFET, SOT-23</t>
@@ -284,7 +293,7 @@
     <t>C2886430</t>
   </si>
   <si>
-    <t>13</t>
+    <t>14</t>
   </si>
   <si>
     <t>Resistor</t>
@@ -305,7 +314,7 @@
     <t>C21189</t>
   </si>
   <si>
-    <t>14</t>
+    <t>15</t>
   </si>
   <si>
     <t>R13 R14</t>
@@ -314,7 +323,7 @@
     <t>R_0603_1608Metric</t>
   </si>
   <si>
-    <t>15</t>
+    <t>16</t>
   </si>
   <si>
     <t>R3 R4</t>
@@ -329,7 +338,7 @@
     <t>C21190</t>
   </si>
   <si>
-    <t>16</t>
+    <t>17</t>
   </si>
   <si>
     <t>R6</t>
@@ -341,7 +350,7 @@
     <t>C22975</t>
   </si>
   <si>
-    <t>17</t>
+    <t>18</t>
   </si>
   <si>
     <t>R8 R15</t>
@@ -353,7 +362,7 @@
     <t>C4190</t>
   </si>
   <si>
-    <t>18</t>
+    <t>19</t>
   </si>
   <si>
     <t>R2</t>
@@ -365,7 +374,7 @@
     <t>C23186</t>
   </si>
   <si>
-    <t>19</t>
+    <t>20</t>
   </si>
   <si>
     <t>R1</t>
@@ -377,7 +386,7 @@
     <t>C25804</t>
   </si>
   <si>
-    <t>20</t>
+    <t>21</t>
   </si>
   <si>
     <t>R7</t>
@@ -389,7 +398,7 @@
     <t>C4184</t>
   </si>
   <si>
-    <t>21</t>
+    <t>22</t>
   </si>
   <si>
     <t>R5</t>
@@ -401,7 +410,7 @@
     <t>C25819</t>
   </si>
   <si>
-    <t>22</t>
+    <t>23</t>
   </si>
   <si>
     <t>Switch, single pole double throw</t>
@@ -419,7 +428,7 @@
     <t>https://www.digikey.jp/ja/products/detail/c-k/OS102011MA1QN1/1981430</t>
   </si>
   <si>
-    <t>23</t>
+    <t>24</t>
   </si>
   <si>
     <t>True RS-485/RS-422, 10Mbps, Slew-Rate Limited, with low-power shutdown, with receiver/driver enable, 32 receiver drive capacitity, DIP-8 and SOIC-8</t>
@@ -461,13 +470,13 @@
     <t>Date:</t>
   </si>
   <si>
-    <t>2023-09-19_04-43-23</t>
+    <t>2026-05-11_13-14-40</t>
   </si>
   <si>
     <t>KiCad Version:</t>
   </si>
   <si>
-    <t>7.0.7-7.0.7~ubuntu23.04.1</t>
+    <t>7.0.11+1</t>
   </si>
   <si>
     <t>Component Groups:</t>
@@ -476,7 +485,7 @@
     <t>Component Count:</t>
   </si>
   <si>
-    <t>33 (27 SMD/ 6 THT)</t>
+    <t>37 (27 SMD/ 10 THT)</t>
   </si>
   <si>
     <t>Fitted Components:</t>
@@ -486,6 +495,9 @@
   </si>
   <si>
     <t>Total Components:</t>
+  </si>
+  <si>
+    <t>Columns colors</t>
   </si>
   <si>
     <t>KiCad Fields (default)</t>
@@ -994,13 +1006,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:K32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
     <col min="2" max="2" width="60.7109375" customWidth="1"/>
     <col min="3" max="3" width="24.7109375" customWidth="1"/>
-    <col min="4" max="4" width="25.7109375" customWidth="1"/>
+    <col min="4" max="4" width="28.7109375" customWidth="1"/>
     <col min="5" max="5" width="24.7109375" customWidth="1"/>
     <col min="6" max="6" width="48.7109375" customWidth="1"/>
     <col min="7" max="7" width="26.7109375" customWidth="1"/>
@@ -1012,7 +1024,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="32" customHeight="1">
       <c r="C1" s="1" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -1025,55 +1037,55 @@
     </row>
     <row r="2" spans="1:11">
       <c r="C2" s="2" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="F2" s="3">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:11">
       <c r="C3" s="2" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="C4" s="2" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>19</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="C5" s="2" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="F5" s="3">
         <v>1</v>
@@ -1081,16 +1093,16 @@
     </row>
     <row r="6" spans="1:11">
       <c r="C6" s="2" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="F6" s="3">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -1268,27 +1280,27 @@
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="30" customHeight="1">
+    <row r="13" spans="1:11">
       <c r="A13" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="D13" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="D13" s="7" t="s">
-        <v>44</v>
-      </c>
       <c r="E13" s="7" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="H13" s="5" t="s">
         <v>17</v>
@@ -1296,31 +1308,31 @@
       <c r="I13" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="J13" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="K13" s="6" t="s">
-        <v>48</v>
+      <c r="J13" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="K13" s="8" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="30" customHeight="1">
       <c r="A14" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="F14" s="11" t="s">
         <v>49</v>
-      </c>
-      <c r="B14" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="F14" s="11" t="s">
-        <v>52</v>
       </c>
       <c r="G14" s="9" t="s">
         <v>11</v>
@@ -1332,33 +1344,33 @@
         <v>18</v>
       </c>
       <c r="J14" s="10" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="K14" s="10" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="30" customHeight="1">
       <c r="A15" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="E15" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="F15" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="C15" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="D15" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>58</v>
-      </c>
       <c r="G15" s="5" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="H15" s="5" t="s">
         <v>17</v>
@@ -1366,34 +1378,34 @@
       <c r="I15" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="J15" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="K15" s="8" t="s">
-        <v>19</v>
+      <c r="J15" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="K15" s="6" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="30" customHeight="1">
       <c r="A16" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="C16" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="D16" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="E16" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="F16" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="D16" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="E16" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="F16" s="11" t="s">
-        <v>63</v>
-      </c>
       <c r="G16" s="9" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="H16" s="9" t="s">
         <v>17</v>
@@ -1401,31 +1413,31 @@
       <c r="I16" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="J16" s="10" t="s">
+      <c r="J16" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="K16" s="12" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="30" customHeight="1">
+      <c r="A17" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C17" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="K16" s="12" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="45" customHeight="1">
-      <c r="A17" s="5" t="s">
+      <c r="D17" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="E17" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="F17" s="7" t="s">
         <v>66</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="E17" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>69</v>
       </c>
       <c r="G17" s="5" t="s">
         <v>11</v>
@@ -1437,7 +1449,7 @@
         <v>18</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="K17" s="8" t="s">
         <v>19</v>
@@ -1445,22 +1457,22 @@
     </row>
     <row r="18" spans="1:11" ht="45" customHeight="1">
       <c r="A18" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="D18" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="B18" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="C18" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="D18" s="11" t="s">
+      <c r="E18" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="F18" s="11" t="s">
         <v>72</v>
-      </c>
-      <c r="E18" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="F18" s="11" t="s">
-        <v>73</v>
       </c>
       <c r="G18" s="9" t="s">
         <v>11</v>
@@ -1471,31 +1483,31 @@
       <c r="I18" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="J18" s="12" t="s">
-        <v>19</v>
+      <c r="J18" s="10" t="s">
+        <v>73</v>
       </c>
       <c r="K18" s="12" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:11">
+    <row r="19" spans="1:11" ht="45" customHeight="1">
       <c r="A19" s="5" t="s">
         <v>74</v>
       </c>
       <c r="B19" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="D19" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="E19" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="F19" s="7" t="s">
         <v>76</v>
-      </c>
-      <c r="D19" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="F19" s="7" t="s">
-        <v>78</v>
       </c>
       <c r="G19" s="5" t="s">
         <v>11</v>
@@ -1503,34 +1515,34 @@
       <c r="H19" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="I19" s="7" t="s">
+      <c r="I19" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="J19" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="K19" s="8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11">
+      <c r="A20" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="C20" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="J19" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="K19" s="6" t="s">
+      <c r="D20" s="11" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" ht="30" customHeight="1">
-      <c r="A20" s="9" t="s">
+      <c r="E20" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="F20" s="11" t="s">
         <v>81</v>
-      </c>
-      <c r="B20" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="C20" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="D20" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="E20" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="F20" s="11" t="s">
-        <v>78</v>
       </c>
       <c r="G20" s="9" t="s">
         <v>11</v>
@@ -1539,71 +1551,71 @@
         <v>17</v>
       </c>
       <c r="I20" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="J20" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="K20" s="10" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="30" customHeight="1">
+      <c r="A21" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B21" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="J20" s="10" t="s">
+      <c r="C21" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="K20" s="10" t="s">
+      <c r="D21" s="7" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="21" spans="1:11">
-      <c r="A21" s="5" t="s">
+      <c r="E21" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="G21" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H21" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I21" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="J21" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="K21" s="6" t="s">
         <v>90</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="E21" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="F21" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="G21" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="H21" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="I21" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="J21" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="K21" s="6" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="D22" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="E22" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="B22" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="C22" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="D22" s="11" t="s">
+      <c r="F22" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="E22" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="F22" s="11" t="s">
-        <v>97</v>
-      </c>
       <c r="G22" s="9" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H22" s="9" t="s">
         <v>17</v>
@@ -1615,27 +1627,27 @@
         <v>19</v>
       </c>
       <c r="K22" s="10" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" ht="30" customHeight="1">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11">
       <c r="A23" s="5" t="s">
         <v>98</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="D23" s="7" t="s">
         <v>99</v>
       </c>
       <c r="E23" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="F23" s="7" t="s">
         <v>100</v>
-      </c>
-      <c r="F23" s="7" t="s">
-        <v>93</v>
       </c>
       <c r="G23" s="5" t="s">
         <v>21</v>
@@ -1646,34 +1658,34 @@
       <c r="I23" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="J23" s="6" t="s">
+      <c r="J23" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="K23" s="6" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="30" customHeight="1">
+      <c r="A24" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="K23" s="6" t="s">
+      <c r="B24" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="D24" s="11" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="24" spans="1:11">
-      <c r="A24" s="9" t="s">
+      <c r="E24" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="B24" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="C24" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="D24" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="E24" s="11" t="s">
-        <v>105</v>
-      </c>
       <c r="F24" s="11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="H24" s="9" t="s">
         <v>17</v>
@@ -1681,34 +1693,34 @@
       <c r="I24" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="J24" s="12" t="s">
-        <v>19</v>
+      <c r="J24" s="10" t="s">
+        <v>104</v>
       </c>
       <c r="K24" s="10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="D25" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="B25" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="C25" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="D25" s="7" t="s">
+      <c r="E25" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="E25" s="7" t="s">
-        <v>109</v>
-      </c>
       <c r="F25" s="7" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="H25" s="5" t="s">
         <v>17</v>
@@ -1720,30 +1732,30 @@
         <v>19</v>
       </c>
       <c r="K25" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="26" spans="1:11">
       <c r="A26" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="D26" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="B26" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="C26" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="D26" s="11" t="s">
+      <c r="E26" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="E26" s="11" t="s">
-        <v>113</v>
-      </c>
       <c r="F26" s="11" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="G26" s="9" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="H26" s="9" t="s">
         <v>17</v>
@@ -1755,27 +1767,27 @@
         <v>19</v>
       </c>
       <c r="K26" s="10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="27" spans="1:11">
       <c r="A27" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="D27" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="B27" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="C27" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="D27" s="7" t="s">
+      <c r="E27" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="E27" s="7" t="s">
-        <v>117</v>
-      </c>
       <c r="F27" s="7" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="G27" s="5" t="s">
         <v>11</v>
@@ -1790,27 +1802,27 @@
         <v>19</v>
       </c>
       <c r="K27" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="28" spans="1:11">
       <c r="A28" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C28" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="D28" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="B28" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="C28" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="D28" s="11" t="s">
+      <c r="E28" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="E28" s="11" t="s">
-        <v>121</v>
-      </c>
       <c r="F28" s="11" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="G28" s="9" t="s">
         <v>11</v>
@@ -1825,27 +1837,27 @@
         <v>19</v>
       </c>
       <c r="K28" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="29" spans="1:11">
       <c r="A29" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="D29" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="B29" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="D29" s="7" t="s">
+      <c r="E29" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="E29" s="7" t="s">
-        <v>125</v>
-      </c>
       <c r="F29" s="7" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="G29" s="5" t="s">
         <v>11</v>
@@ -1860,27 +1872,27 @@
         <v>19</v>
       </c>
       <c r="K29" s="6" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11">
+      <c r="A30" s="9" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="30" spans="1:11" ht="30" customHeight="1">
-      <c r="A30" s="9" t="s">
+      <c r="B30" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C30" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="D30" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="B30" s="10" t="s">
+      <c r="E30" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="C30" s="11" t="s">
-        <v>129</v>
-      </c>
-      <c r="D30" s="11" t="s">
-        <v>130</v>
-      </c>
-      <c r="E30" s="11" t="s">
-        <v>129</v>
-      </c>
       <c r="F30" s="11" t="s">
-        <v>131</v>
+        <v>96</v>
       </c>
       <c r="G30" s="9" t="s">
         <v>11</v>
@@ -1891,31 +1903,31 @@
       <c r="I30" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="J30" s="10" t="s">
+      <c r="J30" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="K30" s="10" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="30" customHeight="1">
+      <c r="A31" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="C31" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="K30" s="12" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" ht="45" customHeight="1">
-      <c r="A31" s="5" t="s">
+      <c r="D31" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="E31" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="F31" s="7" t="s">
         <v>134</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>135</v>
-      </c>
-      <c r="D31" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="E31" s="7" t="s">
-        <v>135</v>
-      </c>
-      <c r="F31" s="7" t="s">
-        <v>137</v>
       </c>
       <c r="G31" s="5" t="s">
         <v>11</v>
@@ -1923,14 +1935,49 @@
       <c r="H31" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="I31" s="7" t="s">
+      <c r="I31" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="J31" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="K31" s="8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="45" customHeight="1">
+      <c r="A32" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="C32" s="11" t="s">
         <v>138</v>
       </c>
-      <c r="J31" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="K31" s="6" t="s">
+      <c r="D32" s="11" t="s">
         <v>139</v>
+      </c>
+      <c r="E32" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="F32" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="G32" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H32" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="I32" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="J32" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="K32" s="10" t="s">
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -1945,30 +1992,35 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="50.7109375" customWidth="1"/>
+    <col min="1" max="1" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
-      <c r="A1" s="7" t="s">
-        <v>156</v>
+      <c r="A1" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="2" spans="1:1">
-      <c r="A2" s="5" t="s">
-        <v>157</v>
+      <c r="A2" s="7" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="3" spans="1:1">
-      <c r="A3" s="6" t="s">
-        <v>158</v>
+      <c r="A3" s="5" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="4" spans="1:1">
-      <c r="A4" s="8" t="s">
-        <v>159</v>
+      <c r="A4" s="6" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" s="8" t="s">
+        <v>163</v>
       </c>
     </row>
   </sheetData>

</xml_diff>